<commit_message>
Toplu veri güncelleme (yerel, 17.07.2026 15:24)
</commit_message>
<xml_diff>
--- a/net rezerv/net_rezerv.xlsx
+++ b/net rezerv/net_rezerv.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O961"/>
+  <dimension ref="A1:O962"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45629,6 +45629,53 @@
         <v>4304109418</v>
       </c>
     </row>
+    <row r="962">
+      <c r="A962" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B962" t="n">
+        <v>46.9253</v>
+      </c>
+      <c r="C962" t="n">
+        <v>166219.719447718</v>
+      </c>
+      <c r="D962" t="n">
+        <v>14656.71816695898</v>
+      </c>
+      <c r="E962" t="n">
+        <v>6311.261813989468</v>
+      </c>
+      <c r="F962" t="n">
+        <v>93591.91591742622</v>
+      </c>
+      <c r="G962" t="n">
+        <v>150</v>
+      </c>
+      <c r="H962" t="n">
+        <v>2819.58958</v>
+      </c>
+      <c r="I962" t="n">
+        <v>-2669.58958</v>
+      </c>
+      <c r="J962" t="n">
+        <v>51659.82354934332</v>
+      </c>
+      <c r="K962" t="n">
+        <v>54329.41312934332</v>
+      </c>
+      <c r="L962" t="n">
+        <v>7799910201</v>
+      </c>
+      <c r="M962" t="n">
+        <v>687770897</v>
+      </c>
+      <c r="N962" t="n">
+        <v>296157854</v>
+      </c>
+      <c r="O962" t="n">
+        <v>4391828732</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Otomatik veri güncelleme (04.09.2026 15:08 UTC)
</commit_message>
<xml_diff>
--- a/net rezerv/net_rezerv.xlsx
+++ b/net rezerv/net_rezerv.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1173"/>
+  <dimension ref="A1:R1174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66144,6 +66144,62 @@
         <v>4984290787</v>
       </c>
     </row>
+    <row r="1174">
+      <c r="A1174" s="1" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B1174" t="n">
+        <v>48.2075</v>
+      </c>
+      <c r="C1174" t="n">
+        <v>186244.3259866203</v>
+      </c>
+      <c r="D1174" t="n">
+        <v>81205.06645231551</v>
+      </c>
+      <c r="E1174" t="n">
+        <v>267449.3924389358</v>
+      </c>
+      <c r="F1174" t="n">
+        <v>57033.03411294923</v>
+      </c>
+      <c r="G1174" t="n">
+        <v>14945.64132137115</v>
+      </c>
+      <c r="H1174" t="n">
+        <v>5941.429881242545</v>
+      </c>
+      <c r="I1174" t="n">
+        <v>104450.4662759944</v>
+      </c>
+      <c r="J1174" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1174" t="n">
+        <v>5064.37621</v>
+      </c>
+      <c r="L1174" t="n">
+        <v>-5064.37621</v>
+      </c>
+      <c r="M1174" t="n">
+        <v>60906.78850801224</v>
+      </c>
+      <c r="N1174" t="n">
+        <v>65971.16471801224</v>
+      </c>
+      <c r="O1174" t="n">
+        <v>8978373345</v>
+      </c>
+      <c r="P1174" t="n">
+        <v>720492004</v>
+      </c>
+      <c r="Q1174" t="n">
+        <v>286421481</v>
+      </c>
+      <c r="R1174" t="n">
+        <v>5035295853</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>